<commit_message>
Code updates, putting in stand by till the next Sylvan.Data.Excel release (v0.4.26) https://github.com/MarkPflug/Sylvan/issues/267
</commit_message>
<xml_diff>
--- a/source/Autossential.Workbook.Tests/Samples/OXML_data.xlsx
+++ b/source/Autossential.Workbook.Tests/Samples/OXML_data.xlsx
@@ -1,17 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<x:workbook xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
-  <x:workbookPr/>
-  <x:bookViews>
-    <x:workbookView windowWidth="28800" windowHeight="12300"/>
-  </x:bookViews>
-  <x:sheets>
-    <x:sheet name="Sheet1" sheetId="2" r:id="rId1"/>
-  </x:sheets>
-  <x:calcPr calcId="191029"/>
-  <x:extLst>
-    <x:ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+  <workbookPr/>
+  <bookViews>
+    <workbookView windowWidth="28800" windowHeight="12300"/>
+  </bookViews>
+  <sheets>
+    <sheet name="Header" sheetId="2" r:id="rId1"/>
+    <sheet name="NoHeader" sheetId="3" r:id="rId2"/>
+    <sheet name="Boolean" sheetId="4" r:id="rId3"/>
+    <sheet name="Template" sheetId="5" r:id="rId4"/>
+    <sheet name="Spread" sheetId="6" r:id="rId5"/>
+    <sheet name="Scattered" sheetId="7" r:id="rId6"/>
+  </sheets>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
         <xcalcf:feature name="microsoft.com:Single"/>
@@ -21,13 +26,13 @@
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
-    </x:ext>
-  </x:extLst>
-</x:workbook>
+    </ext>
+  </extLst>
+</workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="53">
   <si>
     <t>Number1</t>
   </si>
@@ -75,6 +80,161 @@
   </si>
   <si>
     <t>59db02bb</t>
+  </si>
+  <si>
+    <t>Word</t>
+  </si>
+  <si>
+    <t>Formula</t>
+  </si>
+  <si>
+    <t>HOME REMODEL</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="48"/>
+        <color rgb="FF000000"/>
+        <rFont val="Avenir Next LT Pro"/>
+        <charset val="0"/>
+      </rPr>
+      <t>TO-DO</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="48"/>
+        <color rgb="FF000000"/>
+        <rFont val="Avenir Next LT Pro"/>
+        <charset val="0"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="48"/>
+        <color rgb="FF000000"/>
+        <rFont val="Avenir Next LT Pro"/>
+        <charset val="0"/>
+      </rPr>
+      <t>LIST</t>
+    </r>
+  </si>
+  <si>
+    <t>TO BE COMPLETED BY</t>
+  </si>
+  <si>
+    <t>Someone</t>
+  </si>
+  <si>
+    <t>DEADLINE</t>
+  </si>
+  <si>
+    <t>01/31/20XX</t>
+  </si>
+  <si>
+    <t>% Done</t>
+  </si>
+  <si>
+    <t>Phase</t>
+  </si>
+  <si>
+    <t>Due By</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Planning</t>
+  </si>
+  <si>
+    <t>10/dez</t>
+  </si>
+  <si>
+    <t>Research local contractors</t>
+  </si>
+  <si>
+    <t>Preparation</t>
+  </si>
+  <si>
+    <t>Select winning bid</t>
+  </si>
+  <si>
+    <t>Task a</t>
+  </si>
+  <si>
+    <t>Consult</t>
+  </si>
+  <si>
+    <t>Task b</t>
+  </si>
+  <si>
+    <t>Follow-up meeting</t>
+  </si>
+  <si>
+    <t>Task c</t>
+  </si>
+  <si>
+    <t>Sign paperwork</t>
+  </si>
+  <si>
+    <t>Task d</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Avenir Next LT Pro"/>
+        <charset val="0"/>
+      </rPr>
+      <t>Begin work</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Avenir Next LT Pro"/>
+        <charset val="0"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>Paperwork</t>
+  </si>
+  <si>
+    <t>Mail in</t>
+  </si>
+  <si>
+    <t>Complete</t>
+  </si>
+  <si>
+    <t>Inspection</t>
+  </si>
+  <si>
+    <t>Follow-up</t>
+  </si>
+  <si>
+    <t>01/fev</t>
+  </si>
+  <si>
+    <t>Meeting</t>
+  </si>
+  <si>
+    <t>A2</t>
+  </si>
+  <si>
+    <t>C3</t>
+  </si>
+  <si>
+    <t>D3</t>
+  </si>
+  <si>
+    <t>G4</t>
+  </si>
+  <si>
+    <t>E6</t>
   </si>
 </sst>
 </file>
@@ -88,7 +248,13 @@
     <numFmt numFmtId="179" formatCode="_-&quot;R$&quot;\ * #,##0_-;\-&quot;R$&quot;\ * #,##0_-;_-&quot;R$&quot;\ * &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="180" formatCode="dd/mm/yyyy\ h:mm"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="29">
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+    </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -97,10 +263,47 @@
       <charset val="0"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Avenir Next LT Pro"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <sz val="22"/>
+      <color rgb="FF003780"/>
+      <name val="Avenir Next LT Pro"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <sz val="48"/>
+      <color rgb="FF000000"/>
+      <name val="Avenir Next LT Pro"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Avenir Next LT Pro"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFE3525"/>
+      <name val="Avenir Next LT Pro"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Avenir Next LT Pro"/>
+      <charset val="0"/>
+    </font>
+    <font>
       <sz val="10"/>
       <color indexed="8"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -109,7 +312,6 @@
       <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -118,7 +320,6 @@
       <sz val="11"/>
       <color rgb="FF800080"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -126,7 +327,6 @@
       <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -135,7 +335,6 @@
       <sz val="18"/>
       <color theme="3"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -144,7 +343,6 @@
       <sz val="11"/>
       <color rgb="FF7F7F7F"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -153,7 +351,6 @@
       <sz val="15"/>
       <color theme="3"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -162,7 +359,6 @@
       <sz val="13"/>
       <color theme="3"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -171,7 +367,6 @@
       <sz val="11"/>
       <color theme="3"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -179,7 +374,6 @@
       <sz val="11"/>
       <color rgb="FF3F3F76"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -188,7 +382,6 @@
       <sz val="11"/>
       <color rgb="FF3F3F3F"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -197,7 +390,6 @@
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -206,7 +398,6 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -214,7 +405,6 @@
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -223,7 +413,6 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -231,7 +420,6 @@
       <sz val="11"/>
       <color rgb="FF006100"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -239,7 +427,6 @@
       <sz val="11"/>
       <color rgb="FF9C0006"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -247,7 +434,6 @@
       <sz val="11"/>
       <color rgb="FF9C6500"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -255,7 +441,6 @@
       <sz val="11"/>
       <color theme="0"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -263,17 +448,35 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="48"/>
+      <color rgb="FF000000"/>
+      <name val="Avenir Next LT Pro"/>
+      <charset val="0"/>
+    </font>
   </fonts>
-  <fills count="33">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF003780"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -571,154 +774,195 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyBorder="0"/>
-    <xf numFmtId="176" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="180" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="180" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1286,6 +1530,12 @@
   <sheetPr/>
   <dimension ref="A1:F11"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="5"/>
+  <cols>
+    <col min="1" max="3" width="9.85714285714286" customWidth="1"/>
+    <col min="4" max="4" width="17" customWidth="1"/>
+    <col min="5" max="5" width="10.1428571428571" customWidth="1"/>
+    <col min="6" max="6" width="8.85714285714286" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" t="s">
@@ -1317,7 +1567,7 @@
       <c r="C2">
         <v>81847.8</v>
       </c>
-      <c r="D2" s="1">
+      <c r="D2" s="3">
         <v>44996.6670148727</v>
       </c>
       <c r="E2" t="s">
@@ -1337,7 +1587,7 @@
       <c r="C3">
         <v>52317.9</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D3" s="3">
         <v>45182.6670148843</v>
       </c>
       <c r="E3" t="s">
@@ -1357,7 +1607,7 @@
       <c r="C4">
         <v>85773.6</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="3">
         <v>45068.6670148843</v>
       </c>
       <c r="E4" t="s">
@@ -1377,7 +1627,7 @@
       <c r="C5">
         <v>87183</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="3">
         <v>45349.6670148843</v>
       </c>
       <c r="E5" t="s">
@@ -1397,7 +1647,7 @@
       <c r="C6">
         <v>30107.7</v>
       </c>
-      <c r="D6" s="1">
+      <c r="D6" s="3">
         <v>45054.6670148843</v>
       </c>
       <c r="E6" t="s">
@@ -1417,7 +1667,7 @@
       <c r="C7">
         <v>-1908.9</v>
       </c>
-      <c r="D7" s="1">
+      <c r="D7" s="3">
         <v>45167.6670148843</v>
       </c>
       <c r="E7" t="s">
@@ -1437,7 +1687,7 @@
       <c r="C8">
         <v>41974.2</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" s="3">
         <v>44676.6670148843</v>
       </c>
       <c r="E8" t="s">
@@ -1457,7 +1707,7 @@
       <c r="C9">
         <v>128266.2</v>
       </c>
-      <c r="D9" s="1">
+      <c r="D9" s="3">
         <v>45743.6670148843</v>
       </c>
       <c r="E9" t="s">
@@ -1477,7 +1727,7 @@
       <c r="C10">
         <v>133728.3</v>
       </c>
-      <c r="D10" s="1">
+      <c r="D10" s="3">
         <v>45378.6670148843</v>
       </c>
       <c r="E10" t="s">
@@ -1497,7 +1747,7 @@
       <c r="C11">
         <v>125336.7</v>
       </c>
-      <c r="D11" s="1">
+      <c r="D11" s="3">
         <v>45385.6670148843</v>
       </c>
       <c r="E11" t="s">
@@ -1512,4 +1762,928 @@
   <pageSetup paperSize="1" orientation="portrait"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
+  <cols>
+    <col min="1" max="1" width="4.57142857142857" customWidth="1"/>
+    <col min="2" max="2" width="8.57142857142857" customWidth="1"/>
+    <col min="3" max="3" width="9.57142857142857" customWidth="1"/>
+    <col min="4" max="4" width="17" customWidth="1"/>
+    <col min="5" max="5" width="10.1428571428571" customWidth="1"/>
+    <col min="6" max="6" width="6.71428571428571" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1">
+        <v>646</v>
+      </c>
+      <c r="B1">
+        <v>22851</v>
+      </c>
+      <c r="C1">
+        <v>81847.8</v>
+      </c>
+      <c r="D1" s="3">
+        <v>44996.6670148727</v>
+      </c>
+      <c r="E1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2">
+        <v>930</v>
+      </c>
+      <c r="B2">
+        <v>37308</v>
+      </c>
+      <c r="C2">
+        <v>52317.9</v>
+      </c>
+      <c r="D2" s="3">
+        <v>45182.6670148843</v>
+      </c>
+      <c r="E2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3">
+        <v>69</v>
+      </c>
+      <c r="B3">
+        <v>-843</v>
+      </c>
+      <c r="C3">
+        <v>85773.6</v>
+      </c>
+      <c r="D3" s="3">
+        <v>45068.6670148843</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4">
+        <v>138</v>
+      </c>
+      <c r="B4">
+        <v>41271</v>
+      </c>
+      <c r="C4">
+        <v>87183</v>
+      </c>
+      <c r="D4" s="3">
+        <v>45349.6670148843</v>
+      </c>
+      <c r="E4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5">
+        <v>424</v>
+      </c>
+      <c r="B5">
+        <v>-2617.5</v>
+      </c>
+      <c r="C5">
+        <v>30107.7</v>
+      </c>
+      <c r="D5" s="3">
+        <v>45054.6670148843</v>
+      </c>
+      <c r="E5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6">
+        <v>133</v>
+      </c>
+      <c r="B6">
+        <v>33183</v>
+      </c>
+      <c r="C6">
+        <v>-1908.9</v>
+      </c>
+      <c r="D6" s="3">
+        <v>45167.6670148843</v>
+      </c>
+      <c r="E6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7">
+        <v>880</v>
+      </c>
+      <c r="B7">
+        <v>42454.5</v>
+      </c>
+      <c r="C7">
+        <v>41974.2</v>
+      </c>
+      <c r="D7" s="3">
+        <v>44676.6670148843</v>
+      </c>
+      <c r="E7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8">
+        <v>954</v>
+      </c>
+      <c r="B8">
+        <v>35580</v>
+      </c>
+      <c r="C8">
+        <v>128266.2</v>
+      </c>
+      <c r="D8" s="3">
+        <v>45743.6670148843</v>
+      </c>
+      <c r="E8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9">
+        <v>877</v>
+      </c>
+      <c r="B9">
+        <v>25842</v>
+      </c>
+      <c r="C9">
+        <v>133728.3</v>
+      </c>
+      <c r="D9" s="3">
+        <v>45378.6670148843</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10">
+        <v>339</v>
+      </c>
+      <c r="B10">
+        <v>-2322</v>
+      </c>
+      <c r="C10">
+        <v>125336.7</v>
+      </c>
+      <c r="D10" s="3">
+        <v>45385.6670148843</v>
+      </c>
+      <c r="E10" t="s">
+        <v>15</v>
+      </c>
+      <c r="F10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="2" outlineLevelCol="1"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="b">
+        <v>1</v>
+      </c>
+      <c r="B2" t="b">
+        <f>TRUE</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="b">
+        <v>0</v>
+      </c>
+      <c r="B3" t="b">
+        <f>FALSE</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:G17"/>
+  <sheetFormatPr defaultColWidth="71.7142857142857" defaultRowHeight="15" outlineLevelCol="6"/>
+  <cols>
+    <col min="1" max="1" width="9.57142857142857" customWidth="1"/>
+    <col min="2" max="2" width="10.8571428571429" customWidth="1"/>
+    <col min="3" max="3" width="13.7142857142857" customWidth="1"/>
+    <col min="4" max="4" width="10.2857142857143" customWidth="1"/>
+    <col min="5" max="5" width="28.1428571428571" customWidth="1"/>
+    <col min="6" max="6" width="14.5714285714286" customWidth="1"/>
+    <col min="7" max="16384" width="71.7142857142857" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" s="4"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="5"/>
+    </row>
+    <row r="2" ht="27" spans="1:7">
+      <c r="A2" s="4"/>
+      <c r="B2" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="5"/>
+    </row>
+    <row r="3" ht="60" spans="1:7">
+      <c r="A3" s="4"/>
+      <c r="B3" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="5"/>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="4"/>
+      <c r="B4" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="8"/>
+      <c r="D4" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" s="9"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="5"/>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" s="4"/>
+      <c r="B5" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="10"/>
+      <c r="D5" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" s="11"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="5"/>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="4"/>
+      <c r="B6" s="12"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="5"/>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="4"/>
+      <c r="B7" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="4"/>
+      <c r="G7" s="5"/>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" s="4"/>
+      <c r="B8" s="14">
+        <v>1</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="E8" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="F8" s="4"/>
+      <c r="G8" s="5"/>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" s="4"/>
+      <c r="B9" s="14">
+        <v>1</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" s="16">
+        <v>45301</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="F9" s="4"/>
+      <c r="G9" s="5"/>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" s="4"/>
+      <c r="B10" s="14">
+        <v>1</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" s="16">
+        <v>45303</v>
+      </c>
+      <c r="E10" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="F10" s="4"/>
+      <c r="G10" s="5"/>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" s="4"/>
+      <c r="B11" s="14">
+        <v>0.5</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" s="16">
+        <v>45306</v>
+      </c>
+      <c r="E11" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="F11" s="4"/>
+      <c r="G11" s="5"/>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" s="4"/>
+      <c r="B12" s="14">
+        <v>0</v>
+      </c>
+      <c r="C12" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="D12" s="16">
+        <v>45311</v>
+      </c>
+      <c r="E12" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="F12" s="4"/>
+      <c r="G12" s="5"/>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" s="4"/>
+      <c r="B13" s="14">
+        <v>0</v>
+      </c>
+      <c r="C13" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13" s="16">
+        <v>45311</v>
+      </c>
+      <c r="E13" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="F13" s="4"/>
+      <c r="G13" s="5"/>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" s="4"/>
+      <c r="B14" s="14">
+        <v>0</v>
+      </c>
+      <c r="C14" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="D14" s="16">
+        <v>45314</v>
+      </c>
+      <c r="E14" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="F14" s="4"/>
+      <c r="G14" s="5"/>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" s="4"/>
+      <c r="B15" s="14">
+        <v>0</v>
+      </c>
+      <c r="C15" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="D15" s="16">
+        <v>45316</v>
+      </c>
+      <c r="E15" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="F15" s="4"/>
+      <c r="G15" s="5"/>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" s="4"/>
+      <c r="B16" s="14">
+        <v>0</v>
+      </c>
+      <c r="C16" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="D16" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="E16" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="F16" s="4"/>
+      <c r="G16" s="5"/>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" s="4"/>
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="4"/>
+      <c r="G17" s="5"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="D5:E5"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:L11"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="3" width="9.85714285714286" customWidth="1"/>
+    <col min="4" max="4" width="17" customWidth="1"/>
+    <col min="5" max="5" width="10.1428571428571" customWidth="1"/>
+    <col min="6" max="6" width="8.85714285714286" customWidth="1"/>
+    <col min="7" max="7" width="4.57142857142857" customWidth="1"/>
+    <col min="8" max="8" width="8.57142857142857" customWidth="1"/>
+    <col min="9" max="9" width="9.57142857142857" customWidth="1"/>
+    <col min="10" max="10" width="17" customWidth="1"/>
+    <col min="11" max="11" width="10.1428571428571" customWidth="1"/>
+    <col min="12" max="12" width="6.71428571428571" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2">
+        <v>646</v>
+      </c>
+      <c r="B2">
+        <v>22851</v>
+      </c>
+      <c r="C2">
+        <v>81847.8</v>
+      </c>
+      <c r="D2" s="3">
+        <v>44996.6670148727</v>
+      </c>
+      <c r="E2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>646</v>
+      </c>
+      <c r="J2" s="3"/>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3">
+        <v>930</v>
+      </c>
+      <c r="B3">
+        <v>37308</v>
+      </c>
+      <c r="C3">
+        <v>52317.9</v>
+      </c>
+      <c r="D3" s="3">
+        <v>45182.6670148843</v>
+      </c>
+      <c r="E3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" t="b">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>930</v>
+      </c>
+      <c r="J3" s="3"/>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4">
+        <v>69</v>
+      </c>
+      <c r="B4">
+        <v>-843</v>
+      </c>
+      <c r="C4">
+        <v>85773.6</v>
+      </c>
+      <c r="D4" s="3">
+        <v>45068.6670148843</v>
+      </c>
+      <c r="E4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" t="b">
+        <v>1</v>
+      </c>
+      <c r="G4">
+        <v>69</v>
+      </c>
+      <c r="J4" s="3"/>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5">
+        <v>138</v>
+      </c>
+      <c r="B5">
+        <v>41271</v>
+      </c>
+      <c r="C5">
+        <v>87183</v>
+      </c>
+      <c r="D5" s="3">
+        <v>45349.6670148843</v>
+      </c>
+      <c r="E5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <v>138</v>
+      </c>
+      <c r="J5" s="3"/>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6">
+        <v>424</v>
+      </c>
+      <c r="B6">
+        <v>-2617.5</v>
+      </c>
+      <c r="C6">
+        <v>30107.7</v>
+      </c>
+      <c r="D6" s="3">
+        <v>45054.6670148843</v>
+      </c>
+      <c r="E6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>424</v>
+      </c>
+      <c r="J6" s="3"/>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="A7">
+        <v>133</v>
+      </c>
+      <c r="B7">
+        <v>33183</v>
+      </c>
+      <c r="C7">
+        <v>-1908.9</v>
+      </c>
+      <c r="D7" s="3">
+        <v>45167.6670148843</v>
+      </c>
+      <c r="E7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" t="b">
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <v>133</v>
+      </c>
+      <c r="J7" s="3"/>
+    </row>
+    <row r="8" spans="1:12">
+      <c r="A8">
+        <v>880</v>
+      </c>
+      <c r="B8">
+        <v>42454.5</v>
+      </c>
+      <c r="C8">
+        <v>41974.2</v>
+      </c>
+      <c r="D8" s="3">
+        <v>44676.6670148843</v>
+      </c>
+      <c r="E8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" t="b">
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <v>880</v>
+      </c>
+      <c r="J8" s="3">
+        <v>44676.6670148843</v>
+      </c>
+      <c r="K8" t="s">
+        <v>12</v>
+      </c>
+      <c r="L8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="A9">
+        <v>954</v>
+      </c>
+      <c r="B9">
+        <v>35580</v>
+      </c>
+      <c r="C9">
+        <v>128266.2</v>
+      </c>
+      <c r="D9" s="3">
+        <v>45743.6670148843</v>
+      </c>
+      <c r="E9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" t="b">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <v>954</v>
+      </c>
+      <c r="J9" s="3">
+        <v>45743.6670148843</v>
+      </c>
+      <c r="K9" t="s">
+        <v>13</v>
+      </c>
+      <c r="L9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="A10">
+        <v>877</v>
+      </c>
+      <c r="B10">
+        <v>25842</v>
+      </c>
+      <c r="C10">
+        <v>133728.3</v>
+      </c>
+      <c r="D10" s="3">
+        <v>45378.6670148843</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G10">
+        <v>877</v>
+      </c>
+      <c r="J10" s="3">
+        <v>45378.6670148843</v>
+      </c>
+      <c r="K10" t="s">
+        <v>14</v>
+      </c>
+      <c r="L10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="A11">
+        <v>339</v>
+      </c>
+      <c r="B11">
+        <v>-2322</v>
+      </c>
+      <c r="C11">
+        <v>125336.7</v>
+      </c>
+      <c r="D11" s="3">
+        <v>45385.6670148843</v>
+      </c>
+      <c r="E11" t="s">
+        <v>15</v>
+      </c>
+      <c r="F11" t="b">
+        <v>1</v>
+      </c>
+      <c r="G11">
+        <v>339</v>
+      </c>
+      <c r="J11" s="3">
+        <v>45385.6670148843</v>
+      </c>
+      <c r="K11" t="s">
+        <v>15</v>
+      </c>
+      <c r="L11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="5" outlineLevelCol="6"/>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" s="1"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
code updates - boolean/string columns fixes
</commit_message>
<xml_diff>
--- a/source/Autossential.Workbook.Tests/Samples/OXML_data.xlsx
+++ b/source/Autossential.Workbook.Tests/Samples/OXML_data.xlsx
@@ -14,18 +14,20 @@
     <x:sheet name="Template" sheetId="4" state="visible" r:id="rId6"/>
     <x:sheet name="Spread" sheetId="5" state="visible" r:id="rId7"/>
     <x:sheet name="Scattered" sheetId="6" state="visible" r:id="rId8"/>
+    <x:sheet name="NotBoolean" sheetId="7" state="visible" r:id="rId9"/>
+    <x:sheet name="Tables" sheetId="8" state="visible" r:id="rId10"/>
   </x:sheets>
-  <x:calcPr refMode="A1" iterate="false" iterateCount="100" iterateDelta="0.0001"/>
+  <x:calcPr refMode="A1" iterate="false" iterateCount="100" iterateDelta="0.001"/>
   <x:extLst>
     <x:ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
+      <loext:extCalcPr stringRefSyntax="CalcA1"/>
     </x:ext>
   </x:extLst>
 </x:workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="72">
   <si>
     <t xml:space="preserve">Number1</t>
   </si>
@@ -95,8 +97,7 @@
         <sz val="48"/>
         <color rgb="FF000000"/>
         <rFont val="Avenir Next LT Pro"/>
-        <family val="0"/>
-        <charset val="1"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">TO-DO</t>
     </r>
@@ -106,8 +107,7 @@
         <sz val="48"/>
         <color rgb="FF000000"/>
         <rFont val="Avenir Next LT Pro"/>
-        <family val="0"/>
-        <charset val="1"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> </t>
     </r>
@@ -116,8 +116,7 @@
         <sz val="48"/>
         <color rgb="FF000000"/>
         <rFont val="Avenir Next LT Pro"/>
-        <family val="0"/>
-        <charset val="1"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">LIST</t>
     </r>
@@ -220,25 +219,76 @@
   </si>
   <si>
     <t xml:space="preserve">E6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">H</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Y</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">yes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">no</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy\ h:mm"/>
-    <numFmt numFmtId="166" formatCode="0%"/>
-    <numFmt numFmtId="167" formatCode="d/mmm"/>
+    <numFmt numFmtId="166" formatCode="&quot;VERDADEIRO&quot;;&quot;VERDADEIRO&quot;;&quot;FALSO&quot;"/>
+    <numFmt numFmtId="167" formatCode="0%"/>
+    <numFmt numFmtId="168" formatCode="dd/mmm"/>
   </numFmts>
   <fonts count="12">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="0"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -259,63 +309,56 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Avenir Next LT Pro"/>
-      <family val="0"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="22"/>
-      <color rgb="FF003780"/>
+      <color rgb="FF003366"/>
       <name val="Avenir Next LT Pro"/>
-      <family val="0"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="48"/>
       <color rgb="FF000000"/>
       <name val="Avenir Next LT Pro"/>
-      <family val="0"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b val="true"/>
       <sz val="48"/>
       <color rgb="FF000000"/>
       <name val="Avenir Next LT Pro"/>
-      <family val="0"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b val="true"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Avenir Next LT Pro"/>
-      <family val="0"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFE3525"/>
+      <color rgb="FFFF6600"/>
       <name val="Avenir Next LT Pro"/>
-      <family val="0"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b val="true"/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Avenir Next LT Pro"/>
-      <family val="0"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
+      <family val="0"/>
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -324,23 +367,36 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor rgb="FFFFFFFF"/>
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFF5CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF003780"/>
+        <fgColor rgb="FF003366"/>
         <bgColor rgb="FF333399"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF5CE"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
   </borders>
@@ -369,7 +425,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="23">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -378,67 +434,87 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="168" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -471,7 +547,7 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFF2F2F2"/>
+      <rgbColor rgb="FFFFF5CE"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
@@ -498,10 +574,10 @@
       <rgbColor rgb="FF99CC00"/>
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
-      <rgbColor rgb="FFFE3525"/>
+      <rgbColor rgb="FFFF6600"/>
       <rgbColor rgb="FF666699"/>
       <rgbColor rgb="FF969696"/>
-      <rgbColor rgb="FF003780"/>
+      <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF003300"/>
       <rgbColor rgb="FF333300"/>
@@ -515,9 +591,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="LibreOffice">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
@@ -525,46 +601,46 @@
         <a:srgbClr val="ffffff"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="18a303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="0369a3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="a33e03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8e03a3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="c99c00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="c9211e"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000ee"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="800080"/>
+        <a:srgbClr val="551a8b"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme>
@@ -572,58 +648,25 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="35000">
-              <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
           <a:prstDash val="solid"/>
+          <a:miter/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
           <a:prstDash val="solid"/>
+          <a:miter/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
           <a:prstDash val="solid"/>
+          <a:miter/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
@@ -641,48 +684,12 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="40000">
-              <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
@@ -695,12 +702,12 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F11"/>
-  <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.96484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="1" width="9.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="10.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="8.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="1" width="9.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="16.93"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="10.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="8.78"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -950,14 +957,14 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F10"/>
-  <sheetFormatPr defaultColWidth="9.1484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.07421875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="8.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="9.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="10.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="6.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="8.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="9.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="16.93"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="10.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="6.64"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1187,13 +1194,13 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="9.1484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.07421875" defaultRowHeight="15.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="19.61"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11.78"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
@@ -1201,8 +1208,8 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
+    <row r="2" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>18</v>
       </c>
       <c r="B2" s="1" t="b">
@@ -1210,7 +1217,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
         <v>19</v>
       </c>
@@ -1236,260 +1243,261 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G17"/>
-  <sheetFormatPr defaultColWidth="71.71484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="71.640625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="13.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="28.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="13.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10.21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="28.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14.49"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="257" min="7" style="1" width="71.64"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3"/>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="4"/>
-    </row>
-    <row r="2" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3"/>
-      <c r="B2" s="5" t="s">
+      <c r="A1" s="4"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="5"/>
+    </row>
+    <row r="2" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="4"/>
+      <c r="B2" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="4"/>
-    </row>
-    <row r="3" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3"/>
-      <c r="B3" s="6" t="s">
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="5"/>
+    </row>
+    <row r="3" customFormat="false" ht="60" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4"/>
+      <c r="B3" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="4"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="5"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3"/>
-      <c r="B4" s="7" t="s">
+      <c r="A4" s="4"/>
+      <c r="B4" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="8" t="s">
+      <c r="C4" s="8"/>
+      <c r="D4" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="8"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="4"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3"/>
-      <c r="B5" s="9" t="s">
+      <c r="A5" s="4"/>
+      <c r="B5" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="C5" s="9"/>
-      <c r="D5" s="10" t="s">
+      <c r="C5" s="10"/>
+      <c r="D5" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="E5" s="10"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="4"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="5"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3"/>
-      <c r="B6" s="11"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="4"/>
-    </row>
-    <row r="7" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3"/>
-      <c r="B7" s="12" t="s">
+      <c r="A6" s="4"/>
+      <c r="B6" s="12"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="5"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4"/>
+      <c r="B7" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="C7" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="D7" s="12" t="s">
+      <c r="D7" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="E7" s="12" t="s">
+      <c r="E7" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="F7" s="3"/>
-      <c r="G7" s="4"/>
-    </row>
-    <row r="8" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3"/>
-      <c r="B8" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="C8" s="14" t="s">
+      <c r="F7" s="4"/>
+      <c r="G7" s="5"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4"/>
+      <c r="B8" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="E8" s="14" t="s">
+      <c r="E8" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="F8" s="3"/>
-      <c r="G8" s="4"/>
-    </row>
-    <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3"/>
-      <c r="B9" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="C9" s="14" t="s">
+      <c r="F8" s="4"/>
+      <c r="G8" s="5"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4"/>
+      <c r="B9" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="D9" s="15" t="n">
+      <c r="D9" s="17" t="n">
         <v>45301</v>
       </c>
-      <c r="E9" s="14" t="s">
+      <c r="E9" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="F9" s="3"/>
-      <c r="G9" s="4"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="5"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3"/>
-      <c r="B10" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="C10" s="14" t="s">
+      <c r="A10" s="4"/>
+      <c r="B10" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="D10" s="15" t="n">
+      <c r="D10" s="17" t="n">
         <v>45303</v>
       </c>
-      <c r="E10" s="14" t="s">
+      <c r="E10" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="F10" s="3"/>
-      <c r="G10" s="4"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="5"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3"/>
-      <c r="B11" s="13" t="n">
+      <c r="A11" s="4"/>
+      <c r="B11" s="14" t="n">
         <v>0.5</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="C11" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="D11" s="15" t="n">
+      <c r="D11" s="17" t="n">
         <v>45306</v>
       </c>
-      <c r="E11" s="14" t="s">
+      <c r="E11" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="F11" s="3"/>
-      <c r="G11" s="4"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3"/>
-      <c r="B12" s="13" t="n">
+      <c r="A12" s="4"/>
+      <c r="B12" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="C12" s="14" t="s">
+      <c r="C12" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="D12" s="15" t="n">
+      <c r="D12" s="17" t="n">
         <v>45311</v>
       </c>
-      <c r="E12" s="14" t="s">
+      <c r="E12" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="F12" s="3"/>
-      <c r="G12" s="4"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="5"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3"/>
-      <c r="B13" s="13" t="n">
+      <c r="A13" s="4"/>
+      <c r="B13" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="C13" s="14" t="s">
+      <c r="C13" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="D13" s="15" t="n">
+      <c r="D13" s="17" t="n">
         <v>45311</v>
       </c>
-      <c r="E13" s="14" t="s">
+      <c r="E13" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="F13" s="3"/>
-      <c r="G13" s="4"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="5"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3"/>
-      <c r="B14" s="13" t="n">
+      <c r="A14" s="4"/>
+      <c r="B14" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="C14" s="14" t="s">
+      <c r="C14" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="D14" s="15" t="n">
+      <c r="D14" s="17" t="n">
         <v>45314</v>
       </c>
-      <c r="E14" s="14" t="s">
+      <c r="E14" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="F14" s="3"/>
-      <c r="G14" s="4"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="5"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3"/>
-      <c r="B15" s="13" t="n">
+      <c r="A15" s="4"/>
+      <c r="B15" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="C15" s="14" t="s">
+      <c r="C15" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="D15" s="15" t="n">
+      <c r="D15" s="17" t="n">
         <v>45316</v>
       </c>
-      <c r="E15" s="14" t="s">
+      <c r="E15" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="F15" s="3"/>
-      <c r="G15" s="4"/>
+      <c r="F15" s="4"/>
+      <c r="G15" s="5"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3"/>
-      <c r="B16" s="13" t="n">
+      <c r="A16" s="4"/>
+      <c r="B16" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="C16" s="14" t="s">
+      <c r="C16" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="D16" s="9" t="s">
+      <c r="D16" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="E16" s="14" t="s">
+      <c r="E16" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="F16" s="3"/>
-      <c r="G16" s="4"/>
+      <c r="F16" s="4"/>
+      <c r="G16" s="5"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
-      <c r="G17" s="4"/>
+      <c r="A17" s="4"/>
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="4"/>
+      <c r="G17" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1516,18 +1524,18 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L11"/>
-  <sheetFormatPr defaultColWidth="9.1484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.07421875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="1" width="9.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="10.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="8.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="4.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="8.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="9.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="10.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="6.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="1" width="9.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="16.93"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="10.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="8.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="4.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="8.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="9.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="16.93"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="10.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="6.64"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1853,71 +1861,71 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultColWidth="9.1484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.07421875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="16"/>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
+      <c r="A1" s="18"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="16"/>
-      <c r="B3" s="16"/>
-      <c r="C3" s="16" t="s">
+      <c r="A3" s="18"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="D3" s="17" t="s">
+      <c r="D3" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
-      <c r="G3" s="16"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="16"/>
-      <c r="B4" s="16"/>
-      <c r="C4" s="16"/>
-      <c r="D4" s="17"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="16"/>
-      <c r="G4" s="16" t="s">
+      <c r="A4" s="18"/>
+      <c r="B4" s="18"/>
+      <c r="C4" s="18"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="18"/>
+      <c r="F4" s="18"/>
+      <c r="G4" s="18" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="16"/>
-      <c r="B5" s="16"/>
-      <c r="C5" s="16"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="16"/>
-      <c r="G5" s="16"/>
+      <c r="A5" s="18"/>
+      <c r="B5" s="18"/>
+      <c r="C5" s="18"/>
+      <c r="D5" s="19"/>
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="16"/>
-      <c r="B6" s="16"/>
-      <c r="C6" s="16"/>
-      <c r="D6" s="17"/>
-      <c r="E6" s="16" t="s">
+      <c r="A6" s="18"/>
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="19"/>
+      <c r="E6" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="F6" s="16"/>
-      <c r="G6" s="16"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1928,4 +1936,280 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr defaultColWidth="11.5" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="D1" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1" s="20" t="s">
+        <v>60</v>
+      </c>
+      <c r="G1" s="20" t="s">
+        <v>61</v>
+      </c>
+      <c r="H1" s="20" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="20" t="s">
+        <v>63</v>
+      </c>
+      <c r="B2" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="C2" s="20" t="s">
+        <v>65</v>
+      </c>
+      <c r="D2" s="20" t="s">
+        <v>60</v>
+      </c>
+      <c r="E2" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="F2" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="G2" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="H2" s="20" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="20" t="s">
+        <v>63</v>
+      </c>
+      <c r="B3" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="C3" s="20" t="s">
+        <v>65</v>
+      </c>
+      <c r="D3" s="20" t="s">
+        <v>60</v>
+      </c>
+      <c r="E3" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="F3" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="G3" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="H3" s="20" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="20" t="s">
+        <v>63</v>
+      </c>
+      <c r="B4" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="C4" s="20" t="s">
+        <v>65</v>
+      </c>
+      <c r="D4" s="20" t="s">
+        <v>60</v>
+      </c>
+      <c r="E4" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="F4" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="G4" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="H4" s="20" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="20" t="s">
+        <v>63</v>
+      </c>
+      <c r="B5" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="C5" s="20" t="s">
+        <v>65</v>
+      </c>
+      <c r="D5" s="20" t="s">
+        <v>60</v>
+      </c>
+      <c r="E5" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="F5" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="G5" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="H5" s="20" t="s">
+        <v>65</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12ffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12ffffffPágina &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:I6"/>
+  <sheetFormatPr defaultColWidth="11.5234375" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="21" t="s">
+        <v>68</v>
+      </c>
+      <c r="B1" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="C1" s="21" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" s="22" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="B3" s="22" t="n">
+        <v>6</v>
+      </c>
+      <c r="C3" s="22" t="n">
+        <v>7</v>
+      </c>
+      <c r="E3" s="21" t="s">
+        <v>68</v>
+      </c>
+      <c r="F3" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="G3" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="H3" s="21" t="s">
+        <v>70</v>
+      </c>
+      <c r="I3" s="21" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="22" t="n">
+        <v>9</v>
+      </c>
+      <c r="B4" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="C4" s="22" t="n">
+        <v>11</v>
+      </c>
+      <c r="E4" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G4" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="H4" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="I4" s="21" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E5" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>6</v>
+      </c>
+      <c r="G5" s="22" t="n">
+        <v>7</v>
+      </c>
+      <c r="H5" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="I5" s="21" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E6" s="22" t="n">
+        <v>9</v>
+      </c>
+      <c r="F6" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G6" s="22" t="n">
+        <v>11</v>
+      </c>
+      <c r="H6" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="I6" s="21" t="s">
+        <v>63</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12ffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12ffffffPágina &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>